<commit_message>
Mover grid de 6 paquetes de la seccion Hero a la seccion de Diagnostico
</commit_message>
<xml_diff>
--- a/Matriz con Respuestas Expeditas - Consultores NyT.xlsx
+++ b/Matriz con Respuestas Expeditas - Consultores NyT.xlsx
@@ -8,14 +8,27 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emili\OneDrive\Desktop\Developer\Diagnóstico de preguntas revela fugas operativas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53C2DD25-73D0-4FB6-9FED-BA2C4C10FEB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DECFFA40-7A9F-4AF7-947E-F3C25CFC8292}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja2" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -677,7 +690,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -688,6 +701,14 @@
     <font>
       <b/>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
@@ -737,7 +758,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -751,6 +772,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -762,6 +786,9 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1109,23 +1136,31 @@
     <col min="10" max="16384" width="11.19921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" ht="18" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:10" ht="42.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="10" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A3" s="3" t="s">
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
+      <c r="H2" s="10"/>
+      <c r="I2" s="10"/>
+    </row>
+    <row r="3" spans="1:10" ht="18" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:10" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+    <row r="6" spans="1:10" s="5" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>3</v>
       </c>
     </row>
@@ -1145,216 +1180,216 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
+      <c r="A10" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="8" t="s">
+      <c r="B10" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="8" t="s">
+      <c r="C10" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D10" s="8" t="s">
+      <c r="D10" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E10" s="8" t="s">
+      <c r="E10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F10" s="8" t="s">
+      <c r="F10" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G10" s="8" t="s">
+      <c r="G10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="8" t="s">
+      <c r="H10" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="I10" s="8" t="s">
+      <c r="I10" s="9" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="11" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A11" s="6" t="s">
+      <c r="A11" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="F11" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H11" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I11" s="5" t="s">
+      <c r="F11" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J11" s="2"/>
     </row>
     <row r="12" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A12" s="6" t="s">
+      <c r="A12" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="5" t="s">
+      <c r="E12" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F12" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H12" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I12" s="5" t="s">
+      <c r="F12" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I12" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J12" s="2"/>
     </row>
     <row r="13" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="5" t="s">
+      <c r="E13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="F13" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G13" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H13" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I13" s="5" t="s">
+      <c r="F13" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I13" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J13" s="2"/>
     </row>
     <row r="14" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A14" s="6" t="s">
+      <c r="A14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B14" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="E14" s="5" t="s">
+      <c r="E14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="F14" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G14" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H14" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="5" t="s">
+      <c r="F14" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J14" s="2"/>
     </row>
     <row r="15" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A15" s="6" t="s">
+      <c r="A15" s="7" t="s">
         <v>40</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B15" s="6" t="s">
         <v>41</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>42</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>43</v>
       </c>
-      <c r="E15" s="5" t="s">
+      <c r="E15" s="6" t="s">
         <v>44</v>
       </c>
-      <c r="F15" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G15" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H15" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I15" s="5" t="s">
+      <c r="F15" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I15" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10" ht="78" x14ac:dyDescent="0.3">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="B16" s="5" t="s">
+      <c r="B16" s="6" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>48</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="E16" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="F16" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G16" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H16" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I16" s="5" t="s">
+      <c r="F16" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H16" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I16" s="6" t="s">
         <v>24</v>
       </c>
       <c r="J16" s="2"/>
     </row>
     <row r="19" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
+      <c r="A19" s="5" t="s">
         <v>50</v>
       </c>
     </row>
@@ -1374,210 +1409,210 @@
       </c>
     </row>
     <row r="23" spans="1:9" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="6" t="s">
+      <c r="D23" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E23" s="6" t="s">
+      <c r="E23" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F23" s="6" t="s">
+      <c r="F23" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G23" s="6" t="s">
+      <c r="G23" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H23" s="6" t="s">
+      <c r="H23" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I23" s="6" t="s">
+      <c r="I23" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="24" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A24" s="6" t="s">
+      <c r="A24" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="B24" s="5" t="s">
+      <c r="B24" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="E24" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="F24" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G24" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H24" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="5" t="s">
+      <c r="F24" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H24" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="25" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A25" s="6" t="s">
+      <c r="A25" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="B25" s="5" t="s">
+      <c r="B25" s="6" t="s">
         <v>59</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="E25" s="5" t="s">
+      <c r="E25" s="6" t="s">
         <v>62</v>
       </c>
-      <c r="F25" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G25" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H25" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I25" s="5" t="s">
+      <c r="F25" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I25" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A26" s="6" t="s">
+      <c r="A26" s="7" t="s">
         <v>63</v>
       </c>
-      <c r="B26" s="5" t="s">
+      <c r="B26" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="E26" s="5" t="s">
+      <c r="E26" s="6" t="s">
         <v>67</v>
       </c>
-      <c r="F26" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G26" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H26" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I26" s="5" t="s">
+      <c r="F26" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H26" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I26" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="27" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A27" s="6" t="s">
+      <c r="A27" s="7" t="s">
         <v>68</v>
       </c>
-      <c r="B27" s="5" t="s">
+      <c r="B27" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>70</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="E27" s="6" t="s">
         <v>72</v>
       </c>
-      <c r="F27" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G27" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I27" s="5" t="s">
+      <c r="F27" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I27" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A28" s="6" t="s">
+      <c r="A28" s="7" t="s">
         <v>73</v>
       </c>
-      <c r="B28" s="5" t="s">
+      <c r="B28" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>76</v>
       </c>
-      <c r="E28" s="5" t="s">
+      <c r="E28" s="6" t="s">
         <v>77</v>
       </c>
-      <c r="F28" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G28" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H28" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I28" s="5" t="s">
+      <c r="F28" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G28" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H28" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I28" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="29" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="E29" s="5" t="s">
+      <c r="E29" s="6" t="s">
         <v>82</v>
       </c>
-      <c r="F29" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G29" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H29" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I29" s="5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
+      <c r="F29" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" s="5" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="A32" s="5" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1597,210 +1632,210 @@
       </c>
     </row>
     <row r="36" spans="1:9" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A36" s="6" t="s">
+      <c r="A36" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B36" s="6" t="s">
+      <c r="B36" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C36" s="6" t="s">
+      <c r="C36" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D36" s="6" t="s">
+      <c r="D36" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E36" s="6" t="s">
+      <c r="E36" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F36" s="6" t="s">
+      <c r="F36" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G36" s="6" t="s">
+      <c r="G36" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H36" s="6" t="s">
+      <c r="H36" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I36" s="6" t="s">
+      <c r="I36" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="37" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A37" s="6" t="s">
+      <c r="A37" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="B37" s="5" t="s">
+      <c r="B37" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>88</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="E37" s="5" t="s">
+      <c r="E37" s="6" t="s">
         <v>90</v>
       </c>
-      <c r="F37" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G37" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H37" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I37" s="5" t="s">
+      <c r="F37" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G37" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H37" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I37" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="38" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A38" s="6" t="s">
+      <c r="A38" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="B38" s="5" t="s">
+      <c r="B38" s="6" t="s">
         <v>92</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C38" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="6" t="s">
         <v>94</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="E38" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="F38" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G38" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H38" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I38" s="5" t="s">
+      <c r="F38" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G38" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H38" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I38" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="39" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A39" s="6" t="s">
+      <c r="A39" s="7" t="s">
         <v>96</v>
       </c>
-      <c r="B39" s="5" t="s">
+      <c r="B39" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>98</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="E39" s="5" t="s">
+      <c r="E39" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="F39" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G39" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H39" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I39" s="5" t="s">
+      <c r="F39" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G39" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H39" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I39" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="40" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A40" s="6" t="s">
+      <c r="A40" s="7" t="s">
         <v>101</v>
       </c>
-      <c r="B40" s="5" t="s">
+      <c r="B40" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D40" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="E40" s="5" t="s">
+      <c r="E40" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="F40" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G40" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H40" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I40" s="5" t="s">
+      <c r="F40" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G40" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H40" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I40" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="41" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A41" s="6" t="s">
+      <c r="A41" s="7" t="s">
         <v>106</v>
       </c>
-      <c r="B41" s="5" t="s">
+      <c r="B41" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D41" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E41" s="5" t="s">
+      <c r="E41" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="F41" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G41" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H41" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I41" s="5" t="s">
+      <c r="F41" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G41" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H41" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I41" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="42" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A42" s="6" t="s">
+      <c r="A42" s="7" t="s">
         <v>111</v>
       </c>
-      <c r="B42" s="5" t="s">
+      <c r="B42" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="D42" s="5" t="s">
+      <c r="D42" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="E42" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F42" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H42" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I42" s="5" t="s">
+      <c r="F42" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G42" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H42" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I42" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:9" ht="21" x14ac:dyDescent="0.3">
-      <c r="A45" s="4" t="s">
+      <c r="A45" s="5" t="s">
         <v>116</v>
       </c>
     </row>
@@ -1820,210 +1855,210 @@
       </c>
     </row>
     <row r="49" spans="1:9" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A49" s="6" t="s">
+      <c r="A49" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B49" s="6" t="s">
+      <c r="B49" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="C49" s="6" t="s">
+      <c r="C49" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="D49" s="6" t="s">
+      <c r="D49" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="E49" s="6" t="s">
+      <c r="E49" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="F49" s="6" t="s">
+      <c r="F49" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="G49" s="6" t="s">
+      <c r="G49" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="H49" s="6" t="s">
+      <c r="H49" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="I49" s="6" t="s">
+      <c r="I49" s="7" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A50" s="6" t="s">
+      <c r="A50" s="7" t="s">
         <v>119</v>
       </c>
-      <c r="B50" s="5" t="s">
+      <c r="B50" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="C50" s="5" t="s">
+      <c r="C50" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="D50" s="5" t="s">
+      <c r="D50" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="E50" s="5" t="s">
+      <c r="E50" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F50" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G50" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H50" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I50" s="5" t="s">
+      <c r="F50" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G50" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H50" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="51" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A51" s="6" t="s">
+      <c r="A51" s="7" t="s">
         <v>124</v>
       </c>
-      <c r="B51" s="5" t="s">
+      <c r="B51" s="6" t="s">
         <v>125</v>
       </c>
-      <c r="C51" s="5" t="s">
+      <c r="C51" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="D51" s="5" t="s">
+      <c r="D51" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E51" s="5" t="s">
+      <c r="E51" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F51" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G51" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H51" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I51" s="5" t="s">
+      <c r="F51" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G51" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H51" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I51" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A52" s="6" t="s">
+      <c r="A52" s="7" t="s">
         <v>129</v>
       </c>
-      <c r="B52" s="5" t="s">
+      <c r="B52" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="C52" s="5" t="s">
+      <c r="C52" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="D52" s="5" t="s">
+      <c r="D52" s="6" t="s">
         <v>132</v>
       </c>
-      <c r="E52" s="5" t="s">
+      <c r="E52" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F52" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G52" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H52" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I52" s="5" t="s">
+      <c r="F52" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G52" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H52" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I52" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A53" s="6" t="s">
+      <c r="A53" s="7" t="s">
         <v>134</v>
       </c>
-      <c r="B53" s="5" t="s">
+      <c r="B53" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C53" s="5" t="s">
+      <c r="C53" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="D53" s="5" t="s">
+      <c r="D53" s="6" t="s">
         <v>137</v>
       </c>
-      <c r="E53" s="5" t="s">
+      <c r="E53" s="6" t="s">
         <v>138</v>
       </c>
-      <c r="F53" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G53" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H53" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I53" s="5" t="s">
+      <c r="F53" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G53" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H53" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I53" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="54" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A54" s="6" t="s">
+      <c r="A54" s="7" t="s">
         <v>139</v>
       </c>
-      <c r="B54" s="5" t="s">
+      <c r="B54" s="6" t="s">
         <v>140</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="6" t="s">
         <v>141</v>
       </c>
-      <c r="D54" s="5" t="s">
+      <c r="D54" s="6" t="s">
         <v>142</v>
       </c>
-      <c r="E54" s="5" t="s">
+      <c r="E54" s="6" t="s">
         <v>143</v>
       </c>
-      <c r="F54" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G54" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H54" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I54" s="5" t="s">
+      <c r="F54" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H54" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I54" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="55" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A55" s="6" t="s">
+      <c r="A55" s="7" t="s">
         <v>144</v>
       </c>
-      <c r="B55" s="5" t="s">
+      <c r="B55" s="6" t="s">
         <v>145</v>
       </c>
-      <c r="C55" s="5" t="s">
+      <c r="C55" s="6" t="s">
         <v>146</v>
       </c>
-      <c r="D55" s="5" t="s">
+      <c r="D55" s="6" t="s">
         <v>147</v>
       </c>
-      <c r="E55" s="5" t="s">
+      <c r="E55" s="6" t="s">
         <v>148</v>
       </c>
-      <c r="F55" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G55" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="H55" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="I55" s="5" t="s">
+      <c r="F55" s="6" t="s">
+        <v>21</v>
+      </c>
+      <c r="G55" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="H55" s="6" t="s">
+        <v>23</v>
+      </c>
+      <c r="I55" s="6" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="58" spans="1:9" s="3" customFormat="1" ht="21" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
+      <c r="A58" s="5" t="s">
         <v>149</v>
       </c>
     </row>
@@ -2043,210 +2078,210 @@
       </c>
     </row>
     <row r="62" spans="1:9" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A62" s="8" t="s">
+      <c r="A62" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B62" s="8" t="s">
+      <c r="B62" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C62" s="8" t="s">
+      <c r="C62" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D62" s="8" t="s">
+      <c r="D62" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E62" s="8" t="s">
+      <c r="E62" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F62" s="8" t="s">
+      <c r="F62" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G62" s="8" t="s">
+      <c r="G62" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H62" s="8" t="s">
+      <c r="H62" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I62" s="8" t="s">
+      <c r="I62" s="9" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="63" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A63" s="8" t="s">
+      <c r="A63" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="B63" s="7" t="s">
+      <c r="B63" s="8" t="s">
         <v>153</v>
       </c>
-      <c r="C63" s="7" t="s">
+      <c r="C63" s="8" t="s">
         <v>154</v>
       </c>
-      <c r="D63" s="7" t="s">
+      <c r="D63" s="8" t="s">
         <v>155</v>
       </c>
-      <c r="E63" s="7" t="s">
+      <c r="E63" s="8" t="s">
         <v>156</v>
       </c>
-      <c r="F63" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G63" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H63" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I63" s="7" t="s">
+      <c r="F63" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G63" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H63" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I63" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="64" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A64" s="8" t="s">
+      <c r="A64" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B64" s="7" t="s">
+      <c r="B64" s="8" t="s">
         <v>158</v>
       </c>
-      <c r="C64" s="7" t="s">
+      <c r="C64" s="8" t="s">
         <v>159</v>
       </c>
-      <c r="D64" s="7" t="s">
+      <c r="D64" s="8" t="s">
         <v>160</v>
       </c>
-      <c r="E64" s="7" t="s">
+      <c r="E64" s="8" t="s">
         <v>161</v>
       </c>
-      <c r="F64" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G64" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H64" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I64" s="7" t="s">
+      <c r="F64" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G64" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H64" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I64" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A65" s="8" t="s">
+      <c r="A65" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="B65" s="7" t="s">
+      <c r="B65" s="8" t="s">
         <v>163</v>
       </c>
-      <c r="C65" s="7" t="s">
+      <c r="C65" s="8" t="s">
         <v>164</v>
       </c>
-      <c r="D65" s="7" t="s">
+      <c r="D65" s="8" t="s">
         <v>165</v>
       </c>
-      <c r="E65" s="7" t="s">
+      <c r="E65" s="8" t="s">
         <v>166</v>
       </c>
-      <c r="F65" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G65" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H65" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I65" s="7" t="s">
+      <c r="F65" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G65" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H65" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I65" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="66" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A66" s="8" t="s">
+      <c r="A66" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="B66" s="7" t="s">
+      <c r="B66" s="8" t="s">
         <v>168</v>
       </c>
-      <c r="C66" s="7" t="s">
+      <c r="C66" s="8" t="s">
         <v>169</v>
       </c>
-      <c r="D66" s="7" t="s">
+      <c r="D66" s="8" t="s">
         <v>170</v>
       </c>
-      <c r="E66" s="7" t="s">
+      <c r="E66" s="8" t="s">
         <v>171</v>
       </c>
-      <c r="F66" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G66" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H66" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I66" s="7" t="s">
+      <c r="F66" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G66" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H66" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I66" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="67" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A67" s="8" t="s">
+      <c r="A67" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="B67" s="7" t="s">
+      <c r="B67" s="8" t="s">
         <v>173</v>
       </c>
-      <c r="C67" s="7" t="s">
+      <c r="C67" s="8" t="s">
         <v>174</v>
       </c>
-      <c r="D67" s="7" t="s">
+      <c r="D67" s="8" t="s">
         <v>175</v>
       </c>
-      <c r="E67" s="7" t="s">
+      <c r="E67" s="8" t="s">
         <v>176</v>
       </c>
-      <c r="F67" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G67" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H67" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I67" s="7" t="s">
+      <c r="F67" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I67" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A68" s="8" t="s">
+      <c r="A68" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="B68" s="7" t="s">
+      <c r="B68" s="8" t="s">
         <v>178</v>
       </c>
-      <c r="C68" s="7" t="s">
+      <c r="C68" s="8" t="s">
         <v>179</v>
       </c>
-      <c r="D68" s="7" t="s">
+      <c r="D68" s="8" t="s">
         <v>180</v>
       </c>
-      <c r="E68" s="7" t="s">
+      <c r="E68" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="F68" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G68" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H68" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I68" s="7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" s="4" customFormat="1" ht="21" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
+      <c r="F68" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G68" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H68" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I68" s="8" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" s="5" customFormat="1" ht="21" x14ac:dyDescent="0.3">
+      <c r="A71" s="5" t="s">
         <v>182</v>
       </c>
     </row>
@@ -2266,205 +2301,205 @@
       </c>
     </row>
     <row r="75" spans="1:9" s="3" customFormat="1" ht="31.2" x14ac:dyDescent="0.3">
-      <c r="A75" s="8" t="s">
+      <c r="A75" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="B75" s="8" t="s">
+      <c r="B75" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C75" s="8" t="s">
+      <c r="C75" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="D75" s="8" t="s">
+      <c r="D75" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="E75" s="8" t="s">
+      <c r="E75" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="F75" s="8" t="s">
+      <c r="F75" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="G75" s="8" t="s">
+      <c r="G75" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="H75" s="8" t="s">
+      <c r="H75" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="I75" s="8" t="s">
+      <c r="I75" s="9" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A76" s="8" t="s">
+      <c r="A76" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="B76" s="7" t="s">
+      <c r="B76" s="8" t="s">
         <v>186</v>
       </c>
-      <c r="C76" s="7" t="s">
+      <c r="C76" s="8" t="s">
         <v>187</v>
       </c>
-      <c r="D76" s="7" t="s">
+      <c r="D76" s="8" t="s">
         <v>188</v>
       </c>
-      <c r="E76" s="7" t="s">
+      <c r="E76" s="8" t="s">
         <v>189</v>
       </c>
-      <c r="F76" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G76" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H76" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I76" s="7" t="s">
+      <c r="F76" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G76" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H76" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I76" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="77" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A77" s="8" t="s">
+      <c r="A77" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B77" s="7" t="s">
+      <c r="B77" s="8" t="s">
         <v>191</v>
       </c>
-      <c r="C77" s="7" t="s">
+      <c r="C77" s="8" t="s">
         <v>192</v>
       </c>
-      <c r="D77" s="7" t="s">
+      <c r="D77" s="8" t="s">
         <v>193</v>
       </c>
-      <c r="E77" s="7" t="s">
+      <c r="E77" s="8" t="s">
         <v>194</v>
       </c>
-      <c r="F77" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G77" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H77" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I77" s="7" t="s">
+      <c r="F77" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G77" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H77" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I77" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A78" s="8" t="s">
+      <c r="A78" s="9" t="s">
         <v>195</v>
       </c>
-      <c r="B78" s="7" t="s">
+      <c r="B78" s="8" t="s">
         <v>196</v>
       </c>
-      <c r="C78" s="7" t="s">
+      <c r="C78" s="8" t="s">
         <v>197</v>
       </c>
-      <c r="D78" s="7" t="s">
+      <c r="D78" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="E78" s="7" t="s">
+      <c r="E78" s="8" t="s">
         <v>199</v>
       </c>
-      <c r="F78" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G78" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H78" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I78" s="7" t="s">
+      <c r="F78" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H78" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I78" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="79" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A79" s="8" t="s">
+      <c r="A79" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="B79" s="7" t="s">
+      <c r="B79" s="8" t="s">
         <v>201</v>
       </c>
-      <c r="C79" s="7" t="s">
+      <c r="C79" s="8" t="s">
         <v>202</v>
       </c>
-      <c r="D79" s="7" t="s">
+      <c r="D79" s="8" t="s">
         <v>203</v>
       </c>
-      <c r="E79" s="7" t="s">
+      <c r="E79" s="8" t="s">
         <v>204</v>
       </c>
-      <c r="F79" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G79" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H79" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I79" s="7" t="s">
+      <c r="F79" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H79" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I79" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A80" s="8" t="s">
+      <c r="A80" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="B80" s="7" t="s">
+      <c r="B80" s="8" t="s">
         <v>206</v>
       </c>
-      <c r="C80" s="7" t="s">
+      <c r="C80" s="8" t="s">
         <v>207</v>
       </c>
-      <c r="D80" s="7" t="s">
+      <c r="D80" s="8" t="s">
         <v>208</v>
       </c>
-      <c r="E80" s="7" t="s">
+      <c r="E80" s="8" t="s">
         <v>209</v>
       </c>
-      <c r="F80" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G80" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H80" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I80" s="7" t="s">
+      <c r="F80" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G80" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H80" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I80" s="8" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="81" spans="1:9" ht="78" x14ac:dyDescent="0.3">
-      <c r="A81" s="8" t="s">
+      <c r="A81" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B81" s="7" t="s">
+      <c r="B81" s="8" t="s">
         <v>211</v>
       </c>
-      <c r="C81" s="7" t="s">
+      <c r="C81" s="8" t="s">
         <v>212</v>
       </c>
-      <c r="D81" s="7" t="s">
+      <c r="D81" s="8" t="s">
         <v>213</v>
       </c>
-      <c r="E81" s="7" t="s">
+      <c r="E81" s="8" t="s">
         <v>214</v>
       </c>
-      <c r="F81" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="G81" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H81" s="7" t="s">
-        <v>23</v>
-      </c>
-      <c r="I81" s="7" t="s">
+      <c r="F81" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="G81" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="H81" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="I81" s="8" t="s">
         <v>24</v>
       </c>
     </row>
@@ -2479,9 +2514,12 @@
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:I83" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:I1 A4:I83 A2 B3:I3" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>